<commit_message>
Added ERN Studio and Repository
</commit_message>
<xml_diff>
--- a/downloads/citations-per-year-calculator.xlsx
+++ b/downloads/citations-per-year-calculator.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculator" sheetId="1" r:id="R2429031f35544604"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="2" r:id="R7c312c840ed747a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculator" sheetId="1" r:id="R271fae95030a46e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="2" r:id="Rf27053fbcd7c41a6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -820,10 +820,10 @@
         <x:v>Citations Per Year (Now)</x:v>
       </x:c>
       <x:c r="I6" s="44" t="str">
-        <x:v>Citations Per Year (Over Time)</x:v>
+        <x:v>Citations Per Year (Now vs. Lifetime)</x:v>
       </x:c>
       <x:c r="J6" s="44" t="str">
-        <x:v>Citations Per Year (Against stated benchmark)</x:v>
+        <x:v>Citations Per Year (Now vs. Benchmark)</x:v>
       </x:c>
       <x:c r="K6" s="44" t="str">
         <x:v>Plain-English result</x:v>
@@ -867,8 +867,8 @@
         <x:v>1.6666666666666667</x:v>
       </x:c>
       <x:c r="K7" s="56" t="str">
-        <x:f>IF(A7="","",IF(H7="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H7,"0.00")&amp;" citations per year. ")&amp;IF(I7="","Add total citations and publication year for the over-time comparison. ",IF(I7&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I7&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J7="","Name the benchmark and add its annual rate.",IF(J7&gt;1.1,"Against "&amp;F7&amp;": above the benchmark.",IF(J7&lt;0.9,"Against "&amp;F7&amp;": below the benchmark.","Against "&amp;F7&amp;": about the same as the benchmark."))))</x:f>
-        <x:v>Now: 5.00 citations per year. Over time: slower than the paper's lifetime rate. Against 2025 two-year Journal Impact Factor: above the benchmark.</x:v>
+        <x:f>IF(A7="","",IF(H7="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H7,"0.00")&amp;" citations per year. ")&amp;IF(I7="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I7&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I7&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J7="","Name the benchmark and add its annual rate.",IF(J7&gt;1.1,"Now vs. "&amp;F7&amp;": above the benchmark.",IF(J7&lt;0.9,"Now vs. "&amp;F7&amp;": below the benchmark.","Now vs. "&amp;F7&amp;": about the same as the benchmark."))))</x:f>
+        <x:v>Now: 5.00 citations per year. Now vs. lifetime: slower than the paper's lifetime rate. Now vs. 2025 two-year Journal Impact Factor: above the benchmark.</x:v>
       </x:c>
       <x:c r="L7" s="57" t="str">
         <x:v>Google Scholar; 2026-07-28; self-citations included.</x:v>
@@ -892,7 +892,7 @@
         <x:f>IF(OR(A8="",D8="",E8="",F8="",G8="",E8&lt;=0,G8&lt;=0),"",IFERROR(D8/(G8*E8),""))</x:f>
       </x:c>
       <x:c r="K8" s="56" t="str">
-        <x:f>IF(A8="","",IF(H8="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H8,"0.00")&amp;" citations per year. ")&amp;IF(I8="","Add total citations and publication year for the over-time comparison. ",IF(I8&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I8&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J8="","Name the benchmark and add its annual rate.",IF(J8&gt;1.1,"Against "&amp;F8&amp;": above the benchmark.",IF(J8&lt;0.9,"Against "&amp;F8&amp;": below the benchmark.","Against "&amp;F8&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A8="","",IF(H8="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H8,"0.00")&amp;" citations per year. ")&amp;IF(I8="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I8&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I8&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J8="","Name the benchmark and add its annual rate.",IF(J8&gt;1.1,"Now vs. "&amp;F8&amp;": above the benchmark.",IF(J8&lt;0.9,"Now vs. "&amp;F8&amp;": below the benchmark.","Now vs. "&amp;F8&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L8" s="57"/>
     </x:row>
@@ -914,7 +914,7 @@
         <x:f>IF(OR(A9="",D9="",E9="",F9="",G9="",E9&lt;=0,G9&lt;=0),"",IFERROR(D9/(G9*E9),""))</x:f>
       </x:c>
       <x:c r="K9" s="56" t="str">
-        <x:f>IF(A9="","",IF(H9="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H9,"0.00")&amp;" citations per year. ")&amp;IF(I9="","Add total citations and publication year for the over-time comparison. ",IF(I9&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I9&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J9="","Name the benchmark and add its annual rate.",IF(J9&gt;1.1,"Against "&amp;F9&amp;": above the benchmark.",IF(J9&lt;0.9,"Against "&amp;F9&amp;": below the benchmark.","Against "&amp;F9&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A9="","",IF(H9="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H9,"0.00")&amp;" citations per year. ")&amp;IF(I9="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I9&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I9&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J9="","Name the benchmark and add its annual rate.",IF(J9&gt;1.1,"Now vs. "&amp;F9&amp;": above the benchmark.",IF(J9&lt;0.9,"Now vs. "&amp;F9&amp;": below the benchmark.","Now vs. "&amp;F9&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L9" s="57"/>
     </x:row>
@@ -936,7 +936,7 @@
         <x:f>IF(OR(A10="",D10="",E10="",F10="",G10="",E10&lt;=0,G10&lt;=0),"",IFERROR(D10/(G10*E10),""))</x:f>
       </x:c>
       <x:c r="K10" s="56" t="str">
-        <x:f>IF(A10="","",IF(H10="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H10,"0.00")&amp;" citations per year. ")&amp;IF(I10="","Add total citations and publication year for the over-time comparison. ",IF(I10&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I10&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J10="","Name the benchmark and add its annual rate.",IF(J10&gt;1.1,"Against "&amp;F10&amp;": above the benchmark.",IF(J10&lt;0.9,"Against "&amp;F10&amp;": below the benchmark.","Against "&amp;F10&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A10="","",IF(H10="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H10,"0.00")&amp;" citations per year. ")&amp;IF(I10="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I10&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I10&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J10="","Name the benchmark and add its annual rate.",IF(J10&gt;1.1,"Now vs. "&amp;F10&amp;": above the benchmark.",IF(J10&lt;0.9,"Now vs. "&amp;F10&amp;": below the benchmark.","Now vs. "&amp;F10&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L10" s="57"/>
     </x:row>
@@ -958,7 +958,7 @@
         <x:f>IF(OR(A11="",D11="",E11="",F11="",G11="",E11&lt;=0,G11&lt;=0),"",IFERROR(D11/(G11*E11),""))</x:f>
       </x:c>
       <x:c r="K11" s="56" t="str">
-        <x:f>IF(A11="","",IF(H11="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H11,"0.00")&amp;" citations per year. ")&amp;IF(I11="","Add total citations and publication year for the over-time comparison. ",IF(I11&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I11&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J11="","Name the benchmark and add its annual rate.",IF(J11&gt;1.1,"Against "&amp;F11&amp;": above the benchmark.",IF(J11&lt;0.9,"Against "&amp;F11&amp;": below the benchmark.","Against "&amp;F11&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A11="","",IF(H11="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H11,"0.00")&amp;" citations per year. ")&amp;IF(I11="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I11&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I11&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J11="","Name the benchmark and add its annual rate.",IF(J11&gt;1.1,"Now vs. "&amp;F11&amp;": above the benchmark.",IF(J11&lt;0.9,"Now vs. "&amp;F11&amp;": below the benchmark.","Now vs. "&amp;F11&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L11" s="57"/>
     </x:row>
@@ -980,7 +980,7 @@
         <x:f>IF(OR(A12="",D12="",E12="",F12="",G12="",E12&lt;=0,G12&lt;=0),"",IFERROR(D12/(G12*E12),""))</x:f>
       </x:c>
       <x:c r="K12" s="56" t="str">
-        <x:f>IF(A12="","",IF(H12="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H12,"0.00")&amp;" citations per year. ")&amp;IF(I12="","Add total citations and publication year for the over-time comparison. ",IF(I12&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I12&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J12="","Name the benchmark and add its annual rate.",IF(J12&gt;1.1,"Against "&amp;F12&amp;": above the benchmark.",IF(J12&lt;0.9,"Against "&amp;F12&amp;": below the benchmark.","Against "&amp;F12&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A12="","",IF(H12="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H12,"0.00")&amp;" citations per year. ")&amp;IF(I12="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I12&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I12&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J12="","Name the benchmark and add its annual rate.",IF(J12&gt;1.1,"Now vs. "&amp;F12&amp;": above the benchmark.",IF(J12&lt;0.9,"Now vs. "&amp;F12&amp;": below the benchmark.","Now vs. "&amp;F12&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L12" s="57"/>
     </x:row>
@@ -1002,7 +1002,7 @@
         <x:f>IF(OR(A13="",D13="",E13="",F13="",G13="",E13&lt;=0,G13&lt;=0),"",IFERROR(D13/(G13*E13),""))</x:f>
       </x:c>
       <x:c r="K13" s="56" t="str">
-        <x:f>IF(A13="","",IF(H13="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H13,"0.00")&amp;" citations per year. ")&amp;IF(I13="","Add total citations and publication year for the over-time comparison. ",IF(I13&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I13&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J13="","Name the benchmark and add its annual rate.",IF(J13&gt;1.1,"Against "&amp;F13&amp;": above the benchmark.",IF(J13&lt;0.9,"Against "&amp;F13&amp;": below the benchmark.","Against "&amp;F13&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A13="","",IF(H13="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H13,"0.00")&amp;" citations per year. ")&amp;IF(I13="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I13&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I13&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J13="","Name the benchmark and add its annual rate.",IF(J13&gt;1.1,"Now vs. "&amp;F13&amp;": above the benchmark.",IF(J13&lt;0.9,"Now vs. "&amp;F13&amp;": below the benchmark.","Now vs. "&amp;F13&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L13" s="57"/>
     </x:row>
@@ -1024,7 +1024,7 @@
         <x:f>IF(OR(A14="",D14="",E14="",F14="",G14="",E14&lt;=0,G14&lt;=0),"",IFERROR(D14/(G14*E14),""))</x:f>
       </x:c>
       <x:c r="K14" s="56" t="str">
-        <x:f>IF(A14="","",IF(H14="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H14,"0.00")&amp;" citations per year. ")&amp;IF(I14="","Add total citations and publication year for the over-time comparison. ",IF(I14&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I14&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J14="","Name the benchmark and add its annual rate.",IF(J14&gt;1.1,"Against "&amp;F14&amp;": above the benchmark.",IF(J14&lt;0.9,"Against "&amp;F14&amp;": below the benchmark.","Against "&amp;F14&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A14="","",IF(H14="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H14,"0.00")&amp;" citations per year. ")&amp;IF(I14="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I14&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I14&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J14="","Name the benchmark and add its annual rate.",IF(J14&gt;1.1,"Now vs. "&amp;F14&amp;": above the benchmark.",IF(J14&lt;0.9,"Now vs. "&amp;F14&amp;": below the benchmark.","Now vs. "&amp;F14&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L14" s="57"/>
     </x:row>
@@ -1046,7 +1046,7 @@
         <x:f>IF(OR(A15="",D15="",E15="",F15="",G15="",E15&lt;=0,G15&lt;=0),"",IFERROR(D15/(G15*E15),""))</x:f>
       </x:c>
       <x:c r="K15" s="56" t="str">
-        <x:f>IF(A15="","",IF(H15="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H15,"0.00")&amp;" citations per year. ")&amp;IF(I15="","Add total citations and publication year for the over-time comparison. ",IF(I15&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I15&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J15="","Name the benchmark and add its annual rate.",IF(J15&gt;1.1,"Against "&amp;F15&amp;": above the benchmark.",IF(J15&lt;0.9,"Against "&amp;F15&amp;": below the benchmark.","Against "&amp;F15&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A15="","",IF(H15="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H15,"0.00")&amp;" citations per year. ")&amp;IF(I15="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I15&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I15&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J15="","Name the benchmark and add its annual rate.",IF(J15&gt;1.1,"Now vs. "&amp;F15&amp;": above the benchmark.",IF(J15&lt;0.9,"Now vs. "&amp;F15&amp;": below the benchmark.","Now vs. "&amp;F15&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L15" s="57"/>
     </x:row>
@@ -1068,7 +1068,7 @@
         <x:f>IF(OR(A16="",D16="",E16="",F16="",G16="",E16&lt;=0,G16&lt;=0),"",IFERROR(D16/(G16*E16),""))</x:f>
       </x:c>
       <x:c r="K16" s="56" t="str">
-        <x:f>IF(A16="","",IF(H16="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H16,"0.00")&amp;" citations per year. ")&amp;IF(I16="","Add total citations and publication year for the over-time comparison. ",IF(I16&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I16&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J16="","Name the benchmark and add its annual rate.",IF(J16&gt;1.1,"Against "&amp;F16&amp;": above the benchmark.",IF(J16&lt;0.9,"Against "&amp;F16&amp;": below the benchmark.","Against "&amp;F16&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A16="","",IF(H16="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H16,"0.00")&amp;" citations per year. ")&amp;IF(I16="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I16&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I16&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J16="","Name the benchmark and add its annual rate.",IF(J16&gt;1.1,"Now vs. "&amp;F16&amp;": above the benchmark.",IF(J16&lt;0.9,"Now vs. "&amp;F16&amp;": below the benchmark.","Now vs. "&amp;F16&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L16" s="57"/>
     </x:row>
@@ -1090,7 +1090,7 @@
         <x:f>IF(OR(A17="",D17="",E17="",F17="",G17="",E17&lt;=0,G17&lt;=0),"",IFERROR(D17/(G17*E17),""))</x:f>
       </x:c>
       <x:c r="K17" s="56" t="str">
-        <x:f>IF(A17="","",IF(H17="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H17,"0.00")&amp;" citations per year. ")&amp;IF(I17="","Add total citations and publication year for the over-time comparison. ",IF(I17&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I17&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J17="","Name the benchmark and add its annual rate.",IF(J17&gt;1.1,"Against "&amp;F17&amp;": above the benchmark.",IF(J17&lt;0.9,"Against "&amp;F17&amp;": below the benchmark.","Against "&amp;F17&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A17="","",IF(H17="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H17,"0.00")&amp;" citations per year. ")&amp;IF(I17="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I17&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I17&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J17="","Name the benchmark and add its annual rate.",IF(J17&gt;1.1,"Now vs. "&amp;F17&amp;": above the benchmark.",IF(J17&lt;0.9,"Now vs. "&amp;F17&amp;": below the benchmark.","Now vs. "&amp;F17&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L17" s="57"/>
     </x:row>
@@ -1112,7 +1112,7 @@
         <x:f>IF(OR(A18="",D18="",E18="",F18="",G18="",E18&lt;=0,G18&lt;=0),"",IFERROR(D18/(G18*E18),""))</x:f>
       </x:c>
       <x:c r="K18" s="56" t="str">
-        <x:f>IF(A18="","",IF(H18="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H18,"0.00")&amp;" citations per year. ")&amp;IF(I18="","Add total citations and publication year for the over-time comparison. ",IF(I18&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I18&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J18="","Name the benchmark and add its annual rate.",IF(J18&gt;1.1,"Against "&amp;F18&amp;": above the benchmark.",IF(J18&lt;0.9,"Against "&amp;F18&amp;": below the benchmark.","Against "&amp;F18&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A18="","",IF(H18="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H18,"0.00")&amp;" citations per year. ")&amp;IF(I18="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I18&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I18&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J18="","Name the benchmark and add its annual rate.",IF(J18&gt;1.1,"Now vs. "&amp;F18&amp;": above the benchmark.",IF(J18&lt;0.9,"Now vs. "&amp;F18&amp;": below the benchmark.","Now vs. "&amp;F18&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L18" s="57"/>
     </x:row>
@@ -1134,7 +1134,7 @@
         <x:f>IF(OR(A19="",D19="",E19="",F19="",G19="",E19&lt;=0,G19&lt;=0),"",IFERROR(D19/(G19*E19),""))</x:f>
       </x:c>
       <x:c r="K19" s="56" t="str">
-        <x:f>IF(A19="","",IF(H19="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H19,"0.00")&amp;" citations per year. ")&amp;IF(I19="","Add total citations and publication year for the over-time comparison. ",IF(I19&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I19&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J19="","Name the benchmark and add its annual rate.",IF(J19&gt;1.1,"Against "&amp;F19&amp;": above the benchmark.",IF(J19&lt;0.9,"Against "&amp;F19&amp;": below the benchmark.","Against "&amp;F19&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A19="","",IF(H19="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H19,"0.00")&amp;" citations per year. ")&amp;IF(I19="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I19&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I19&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J19="","Name the benchmark and add its annual rate.",IF(J19&gt;1.1,"Now vs. "&amp;F19&amp;": above the benchmark.",IF(J19&lt;0.9,"Now vs. "&amp;F19&amp;": below the benchmark.","Now vs. "&amp;F19&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L19" s="57"/>
     </x:row>
@@ -1156,7 +1156,7 @@
         <x:f>IF(OR(A20="",D20="",E20="",F20="",G20="",E20&lt;=0,G20&lt;=0),"",IFERROR(D20/(G20*E20),""))</x:f>
       </x:c>
       <x:c r="K20" s="56" t="str">
-        <x:f>IF(A20="","",IF(H20="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H20,"0.00")&amp;" citations per year. ")&amp;IF(I20="","Add total citations and publication year for the over-time comparison. ",IF(I20&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I20&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J20="","Name the benchmark and add its annual rate.",IF(J20&gt;1.1,"Against "&amp;F20&amp;": above the benchmark.",IF(J20&lt;0.9,"Against "&amp;F20&amp;": below the benchmark.","Against "&amp;F20&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A20="","",IF(H20="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H20,"0.00")&amp;" citations per year. ")&amp;IF(I20="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I20&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I20&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J20="","Name the benchmark and add its annual rate.",IF(J20&gt;1.1,"Now vs. "&amp;F20&amp;": above the benchmark.",IF(J20&lt;0.9,"Now vs. "&amp;F20&amp;": below the benchmark.","Now vs. "&amp;F20&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L20" s="57"/>
     </x:row>
@@ -1178,7 +1178,7 @@
         <x:f>IF(OR(A21="",D21="",E21="",F21="",G21="",E21&lt;=0,G21&lt;=0),"",IFERROR(D21/(G21*E21),""))</x:f>
       </x:c>
       <x:c r="K21" s="56" t="str">
-        <x:f>IF(A21="","",IF(H21="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H21,"0.00")&amp;" citations per year. ")&amp;IF(I21="","Add total citations and publication year for the over-time comparison. ",IF(I21&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I21&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J21="","Name the benchmark and add its annual rate.",IF(J21&gt;1.1,"Against "&amp;F21&amp;": above the benchmark.",IF(J21&lt;0.9,"Against "&amp;F21&amp;": below the benchmark.","Against "&amp;F21&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A21="","",IF(H21="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H21,"0.00")&amp;" citations per year. ")&amp;IF(I21="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I21&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I21&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J21="","Name the benchmark and add its annual rate.",IF(J21&gt;1.1,"Now vs. "&amp;F21&amp;": above the benchmark.",IF(J21&lt;0.9,"Now vs. "&amp;F21&amp;": below the benchmark.","Now vs. "&amp;F21&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L21" s="57"/>
     </x:row>
@@ -1200,7 +1200,7 @@
         <x:f>IF(OR(A22="",D22="",E22="",F22="",G22="",E22&lt;=0,G22&lt;=0),"",IFERROR(D22/(G22*E22),""))</x:f>
       </x:c>
       <x:c r="K22" s="56" t="str">
-        <x:f>IF(A22="","",IF(H22="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H22,"0.00")&amp;" citations per year. ")&amp;IF(I22="","Add total citations and publication year for the over-time comparison. ",IF(I22&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I22&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J22="","Name the benchmark and add its annual rate.",IF(J22&gt;1.1,"Against "&amp;F22&amp;": above the benchmark.",IF(J22&lt;0.9,"Against "&amp;F22&amp;": below the benchmark.","Against "&amp;F22&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A22="","",IF(H22="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H22,"0.00")&amp;" citations per year. ")&amp;IF(I22="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I22&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I22&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J22="","Name the benchmark and add its annual rate.",IF(J22&gt;1.1,"Now vs. "&amp;F22&amp;": above the benchmark.",IF(J22&lt;0.9,"Now vs. "&amp;F22&amp;": below the benchmark.","Now vs. "&amp;F22&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L22" s="57"/>
     </x:row>
@@ -1222,7 +1222,7 @@
         <x:f>IF(OR(A23="",D23="",E23="",F23="",G23="",E23&lt;=0,G23&lt;=0),"",IFERROR(D23/(G23*E23),""))</x:f>
       </x:c>
       <x:c r="K23" s="56" t="str">
-        <x:f>IF(A23="","",IF(H23="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H23,"0.00")&amp;" citations per year. ")&amp;IF(I23="","Add total citations and publication year for the over-time comparison. ",IF(I23&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I23&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J23="","Name the benchmark and add its annual rate.",IF(J23&gt;1.1,"Against "&amp;F23&amp;": above the benchmark.",IF(J23&lt;0.9,"Against "&amp;F23&amp;": below the benchmark.","Against "&amp;F23&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A23="","",IF(H23="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H23,"0.00")&amp;" citations per year. ")&amp;IF(I23="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I23&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I23&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J23="","Name the benchmark and add its annual rate.",IF(J23&gt;1.1,"Now vs. "&amp;F23&amp;": above the benchmark.",IF(J23&lt;0.9,"Now vs. "&amp;F23&amp;": below the benchmark.","Now vs. "&amp;F23&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L23" s="57"/>
     </x:row>
@@ -1244,7 +1244,7 @@
         <x:f>IF(OR(A24="",D24="",E24="",F24="",G24="",E24&lt;=0,G24&lt;=0),"",IFERROR(D24/(G24*E24),""))</x:f>
       </x:c>
       <x:c r="K24" s="56" t="str">
-        <x:f>IF(A24="","",IF(H24="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H24,"0.00")&amp;" citations per year. ")&amp;IF(I24="","Add total citations and publication year for the over-time comparison. ",IF(I24&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I24&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J24="","Name the benchmark and add its annual rate.",IF(J24&gt;1.1,"Against "&amp;F24&amp;": above the benchmark.",IF(J24&lt;0.9,"Against "&amp;F24&amp;": below the benchmark.","Against "&amp;F24&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A24="","",IF(H24="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H24,"0.00")&amp;" citations per year. ")&amp;IF(I24="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I24&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I24&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J24="","Name the benchmark and add its annual rate.",IF(J24&gt;1.1,"Now vs. "&amp;F24&amp;": above the benchmark.",IF(J24&lt;0.9,"Now vs. "&amp;F24&amp;": below the benchmark.","Now vs. "&amp;F24&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L24" s="57"/>
     </x:row>
@@ -1266,7 +1266,7 @@
         <x:f>IF(OR(A25="",D25="",E25="",F25="",G25="",E25&lt;=0,G25&lt;=0),"",IFERROR(D25/(G25*E25),""))</x:f>
       </x:c>
       <x:c r="K25" s="56" t="str">
-        <x:f>IF(A25="","",IF(H25="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H25,"0.00")&amp;" citations per year. ")&amp;IF(I25="","Add total citations and publication year for the over-time comparison. ",IF(I25&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I25&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J25="","Name the benchmark and add its annual rate.",IF(J25&gt;1.1,"Against "&amp;F25&amp;": above the benchmark.",IF(J25&lt;0.9,"Against "&amp;F25&amp;": below the benchmark.","Against "&amp;F25&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A25="","",IF(H25="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H25,"0.00")&amp;" citations per year. ")&amp;IF(I25="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I25&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I25&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J25="","Name the benchmark and add its annual rate.",IF(J25&gt;1.1,"Now vs. "&amp;F25&amp;": above the benchmark.",IF(J25&lt;0.9,"Now vs. "&amp;F25&amp;": below the benchmark.","Now vs. "&amp;F25&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L25" s="57"/>
     </x:row>
@@ -1288,7 +1288,7 @@
         <x:f>IF(OR(A26="",D26="",E26="",F26="",G26="",E26&lt;=0,G26&lt;=0),"",IFERROR(D26/(G26*E26),""))</x:f>
       </x:c>
       <x:c r="K26" s="56" t="str">
-        <x:f>IF(A26="","",IF(H26="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H26,"0.00")&amp;" citations per year. ")&amp;IF(I26="","Add total citations and publication year for the over-time comparison. ",IF(I26&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I26&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J26="","Name the benchmark and add its annual rate.",IF(J26&gt;1.1,"Against "&amp;F26&amp;": above the benchmark.",IF(J26&lt;0.9,"Against "&amp;F26&amp;": below the benchmark.","Against "&amp;F26&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A26="","",IF(H26="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H26,"0.00")&amp;" citations per year. ")&amp;IF(I26="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I26&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I26&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J26="","Name the benchmark and add its annual rate.",IF(J26&gt;1.1,"Now vs. "&amp;F26&amp;": above the benchmark.",IF(J26&lt;0.9,"Now vs. "&amp;F26&amp;": below the benchmark.","Now vs. "&amp;F26&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L26" s="57"/>
     </x:row>
@@ -1310,7 +1310,7 @@
         <x:f>IF(OR(A27="",D27="",E27="",F27="",G27="",E27&lt;=0,G27&lt;=0),"",IFERROR(D27/(G27*E27),""))</x:f>
       </x:c>
       <x:c r="K27" s="56" t="str">
-        <x:f>IF(A27="","",IF(H27="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H27,"0.00")&amp;" citations per year. ")&amp;IF(I27="","Add total citations and publication year for the over-time comparison. ",IF(I27&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I27&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J27="","Name the benchmark and add its annual rate.",IF(J27&gt;1.1,"Against "&amp;F27&amp;": above the benchmark.",IF(J27&lt;0.9,"Against "&amp;F27&amp;": below the benchmark.","Against "&amp;F27&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A27="","",IF(H27="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H27,"0.00")&amp;" citations per year. ")&amp;IF(I27="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I27&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I27&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J27="","Name the benchmark and add its annual rate.",IF(J27&gt;1.1,"Now vs. "&amp;F27&amp;": above the benchmark.",IF(J27&lt;0.9,"Now vs. "&amp;F27&amp;": below the benchmark.","Now vs. "&amp;F27&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L27" s="57"/>
     </x:row>
@@ -1332,7 +1332,7 @@
         <x:f>IF(OR(A28="",D28="",E28="",F28="",G28="",E28&lt;=0,G28&lt;=0),"",IFERROR(D28/(G28*E28),""))</x:f>
       </x:c>
       <x:c r="K28" s="56" t="str">
-        <x:f>IF(A28="","",IF(H28="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H28,"0.00")&amp;" citations per year. ")&amp;IF(I28="","Add total citations and publication year for the over-time comparison. ",IF(I28&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I28&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J28="","Name the benchmark and add its annual rate.",IF(J28&gt;1.1,"Against "&amp;F28&amp;": above the benchmark.",IF(J28&lt;0.9,"Against "&amp;F28&amp;": below the benchmark.","Against "&amp;F28&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A28="","",IF(H28="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H28,"0.00")&amp;" citations per year. ")&amp;IF(I28="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I28&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I28&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J28="","Name the benchmark and add its annual rate.",IF(J28&gt;1.1,"Now vs. "&amp;F28&amp;": above the benchmark.",IF(J28&lt;0.9,"Now vs. "&amp;F28&amp;": below the benchmark.","Now vs. "&amp;F28&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L28" s="57"/>
     </x:row>
@@ -1354,7 +1354,7 @@
         <x:f>IF(OR(A29="",D29="",E29="",F29="",G29="",E29&lt;=0,G29&lt;=0),"",IFERROR(D29/(G29*E29),""))</x:f>
       </x:c>
       <x:c r="K29" s="56" t="str">
-        <x:f>IF(A29="","",IF(H29="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H29,"0.00")&amp;" citations per year. ")&amp;IF(I29="","Add total citations and publication year for the over-time comparison. ",IF(I29&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I29&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J29="","Name the benchmark and add its annual rate.",IF(J29&gt;1.1,"Against "&amp;F29&amp;": above the benchmark.",IF(J29&lt;0.9,"Against "&amp;F29&amp;": below the benchmark.","Against "&amp;F29&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A29="","",IF(H29="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H29,"0.00")&amp;" citations per year. ")&amp;IF(I29="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I29&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I29&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J29="","Name the benchmark and add its annual rate.",IF(J29&gt;1.1,"Now vs. "&amp;F29&amp;": above the benchmark.",IF(J29&lt;0.9,"Now vs. "&amp;F29&amp;": below the benchmark.","Now vs. "&amp;F29&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L29" s="57"/>
     </x:row>
@@ -1376,7 +1376,7 @@
         <x:f>IF(OR(A30="",D30="",E30="",F30="",G30="",E30&lt;=0,G30&lt;=0),"",IFERROR(D30/(G30*E30),""))</x:f>
       </x:c>
       <x:c r="K30" s="56" t="str">
-        <x:f>IF(A30="","",IF(H30="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H30,"0.00")&amp;" citations per year. ")&amp;IF(I30="","Add total citations and publication year for the over-time comparison. ",IF(I30&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I30&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J30="","Name the benchmark and add its annual rate.",IF(J30&gt;1.1,"Against "&amp;F30&amp;": above the benchmark.",IF(J30&lt;0.9,"Against "&amp;F30&amp;": below the benchmark.","Against "&amp;F30&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A30="","",IF(H30="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H30,"0.00")&amp;" citations per year. ")&amp;IF(I30="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I30&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I30&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J30="","Name the benchmark and add its annual rate.",IF(J30&gt;1.1,"Now vs. "&amp;F30&amp;": above the benchmark.",IF(J30&lt;0.9,"Now vs. "&amp;F30&amp;": below the benchmark.","Now vs. "&amp;F30&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L30" s="57"/>
     </x:row>
@@ -1398,7 +1398,7 @@
         <x:f>IF(OR(A31="",D31="",E31="",F31="",G31="",E31&lt;=0,G31&lt;=0),"",IFERROR(D31/(G31*E31),""))</x:f>
       </x:c>
       <x:c r="K31" s="56" t="str">
-        <x:f>IF(A31="","",IF(H31="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H31,"0.00")&amp;" citations per year. ")&amp;IF(I31="","Add total citations and publication year for the over-time comparison. ",IF(I31&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I31&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J31="","Name the benchmark and add its annual rate.",IF(J31&gt;1.1,"Against "&amp;F31&amp;": above the benchmark.",IF(J31&lt;0.9,"Against "&amp;F31&amp;": below the benchmark.","Against "&amp;F31&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A31="","",IF(H31="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H31,"0.00")&amp;" citations per year. ")&amp;IF(I31="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I31&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I31&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J31="","Name the benchmark and add its annual rate.",IF(J31&gt;1.1,"Now vs. "&amp;F31&amp;": above the benchmark.",IF(J31&lt;0.9,"Now vs. "&amp;F31&amp;": below the benchmark.","Now vs. "&amp;F31&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L31" s="57"/>
     </x:row>
@@ -1420,7 +1420,7 @@
         <x:f>IF(OR(A32="",D32="",E32="",F32="",G32="",E32&lt;=0,G32&lt;=0),"",IFERROR(D32/(G32*E32),""))</x:f>
       </x:c>
       <x:c r="K32" s="56" t="str">
-        <x:f>IF(A32="","",IF(H32="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H32,"0.00")&amp;" citations per year. ")&amp;IF(I32="","Add total citations and publication year for the over-time comparison. ",IF(I32&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I32&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J32="","Name the benchmark and add its annual rate.",IF(J32&gt;1.1,"Against "&amp;F32&amp;": above the benchmark.",IF(J32&lt;0.9,"Against "&amp;F32&amp;": below the benchmark.","Against "&amp;F32&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A32="","",IF(H32="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H32,"0.00")&amp;" citations per year. ")&amp;IF(I32="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I32&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I32&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J32="","Name the benchmark and add its annual rate.",IF(J32&gt;1.1,"Now vs. "&amp;F32&amp;": above the benchmark.",IF(J32&lt;0.9,"Now vs. "&amp;F32&amp;": below the benchmark.","Now vs. "&amp;F32&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L32" s="57"/>
     </x:row>
@@ -1442,7 +1442,7 @@
         <x:f>IF(OR(A33="",D33="",E33="",F33="",G33="",E33&lt;=0,G33&lt;=0),"",IFERROR(D33/(G33*E33),""))</x:f>
       </x:c>
       <x:c r="K33" s="56" t="str">
-        <x:f>IF(A33="","",IF(H33="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H33,"0.00")&amp;" citations per year. ")&amp;IF(I33="","Add total citations and publication year for the over-time comparison. ",IF(I33&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I33&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J33="","Name the benchmark and add its annual rate.",IF(J33&gt;1.1,"Against "&amp;F33&amp;": above the benchmark.",IF(J33&lt;0.9,"Against "&amp;F33&amp;": below the benchmark.","Against "&amp;F33&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A33="","",IF(H33="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H33,"0.00")&amp;" citations per year. ")&amp;IF(I33="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I33&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I33&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J33="","Name the benchmark and add its annual rate.",IF(J33&gt;1.1,"Now vs. "&amp;F33&amp;": above the benchmark.",IF(J33&lt;0.9,"Now vs. "&amp;F33&amp;": below the benchmark.","Now vs. "&amp;F33&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L33" s="57"/>
     </x:row>
@@ -1464,7 +1464,7 @@
         <x:f>IF(OR(A34="",D34="",E34="",F34="",G34="",E34&lt;=0,G34&lt;=0),"",IFERROR(D34/(G34*E34),""))</x:f>
       </x:c>
       <x:c r="K34" s="56" t="str">
-        <x:f>IF(A34="","",IF(H34="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H34,"0.00")&amp;" citations per year. ")&amp;IF(I34="","Add total citations and publication year for the over-time comparison. ",IF(I34&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I34&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J34="","Name the benchmark and add its annual rate.",IF(J34&gt;1.1,"Against "&amp;F34&amp;": above the benchmark.",IF(J34&lt;0.9,"Against "&amp;F34&amp;": below the benchmark.","Against "&amp;F34&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A34="","",IF(H34="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H34,"0.00")&amp;" citations per year. ")&amp;IF(I34="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I34&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I34&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J34="","Name the benchmark and add its annual rate.",IF(J34&gt;1.1,"Now vs. "&amp;F34&amp;": above the benchmark.",IF(J34&lt;0.9,"Now vs. "&amp;F34&amp;": below the benchmark.","Now vs. "&amp;F34&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L34" s="57"/>
     </x:row>
@@ -1486,7 +1486,7 @@
         <x:f>IF(OR(A35="",D35="",E35="",F35="",G35="",E35&lt;=0,G35&lt;=0),"",IFERROR(D35/(G35*E35),""))</x:f>
       </x:c>
       <x:c r="K35" s="56" t="str">
-        <x:f>IF(A35="","",IF(H35="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H35,"0.00")&amp;" citations per year. ")&amp;IF(I35="","Add total citations and publication year for the over-time comparison. ",IF(I35&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I35&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J35="","Name the benchmark and add its annual rate.",IF(J35&gt;1.1,"Against "&amp;F35&amp;": above the benchmark.",IF(J35&lt;0.9,"Against "&amp;F35&amp;": below the benchmark.","Against "&amp;F35&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A35="","",IF(H35="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H35,"0.00")&amp;" citations per year. ")&amp;IF(I35="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I35&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I35&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J35="","Name the benchmark and add its annual rate.",IF(J35&gt;1.1,"Now vs. "&amp;F35&amp;": above the benchmark.",IF(J35&lt;0.9,"Now vs. "&amp;F35&amp;": below the benchmark.","Now vs. "&amp;F35&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L35" s="57"/>
     </x:row>
@@ -1508,7 +1508,7 @@
         <x:f>IF(OR(A36="",D36="",E36="",F36="",G36="",E36&lt;=0,G36&lt;=0),"",IFERROR(D36/(G36*E36),""))</x:f>
       </x:c>
       <x:c r="K36" s="56" t="str">
-        <x:f>IF(A36="","",IF(H36="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H36,"0.00")&amp;" citations per year. ")&amp;IF(I36="","Add total citations and publication year for the over-time comparison. ",IF(I36&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I36&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J36="","Name the benchmark and add its annual rate.",IF(J36&gt;1.1,"Against "&amp;F36&amp;": above the benchmark.",IF(J36&lt;0.9,"Against "&amp;F36&amp;": below the benchmark.","Against "&amp;F36&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A36="","",IF(H36="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H36,"0.00")&amp;" citations per year. ")&amp;IF(I36="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I36&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I36&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J36="","Name the benchmark and add its annual rate.",IF(J36&gt;1.1,"Now vs. "&amp;F36&amp;": above the benchmark.",IF(J36&lt;0.9,"Now vs. "&amp;F36&amp;": below the benchmark.","Now vs. "&amp;F36&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L36" s="57"/>
     </x:row>
@@ -1530,7 +1530,7 @@
         <x:f>IF(OR(A37="",D37="",E37="",F37="",G37="",E37&lt;=0,G37&lt;=0),"",IFERROR(D37/(G37*E37),""))</x:f>
       </x:c>
       <x:c r="K37" s="56" t="str">
-        <x:f>IF(A37="","",IF(H37="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H37,"0.00")&amp;" citations per year. ")&amp;IF(I37="","Add total citations and publication year for the over-time comparison. ",IF(I37&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I37&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J37="","Name the benchmark and add its annual rate.",IF(J37&gt;1.1,"Against "&amp;F37&amp;": above the benchmark.",IF(J37&lt;0.9,"Against "&amp;F37&amp;": below the benchmark.","Against "&amp;F37&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A37="","",IF(H37="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H37,"0.00")&amp;" citations per year. ")&amp;IF(I37="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I37&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I37&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J37="","Name the benchmark and add its annual rate.",IF(J37&gt;1.1,"Now vs. "&amp;F37&amp;": above the benchmark.",IF(J37&lt;0.9,"Now vs. "&amp;F37&amp;": below the benchmark.","Now vs. "&amp;F37&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L37" s="57"/>
     </x:row>
@@ -1552,7 +1552,7 @@
         <x:f>IF(OR(A38="",D38="",E38="",F38="",G38="",E38&lt;=0,G38&lt;=0),"",IFERROR(D38/(G38*E38),""))</x:f>
       </x:c>
       <x:c r="K38" s="56" t="str">
-        <x:f>IF(A38="","",IF(H38="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H38,"0.00")&amp;" citations per year. ")&amp;IF(I38="","Add total citations and publication year for the over-time comparison. ",IF(I38&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I38&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J38="","Name the benchmark and add its annual rate.",IF(J38&gt;1.1,"Against "&amp;F38&amp;": above the benchmark.",IF(J38&lt;0.9,"Against "&amp;F38&amp;": below the benchmark.","Against "&amp;F38&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A38="","",IF(H38="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H38,"0.00")&amp;" citations per year. ")&amp;IF(I38="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I38&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I38&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J38="","Name the benchmark and add its annual rate.",IF(J38&gt;1.1,"Now vs. "&amp;F38&amp;": above the benchmark.",IF(J38&lt;0.9,"Now vs. "&amp;F38&amp;": below the benchmark.","Now vs. "&amp;F38&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L38" s="57"/>
     </x:row>
@@ -1574,7 +1574,7 @@
         <x:f>IF(OR(A39="",D39="",E39="",F39="",G39="",E39&lt;=0,G39&lt;=0),"",IFERROR(D39/(G39*E39),""))</x:f>
       </x:c>
       <x:c r="K39" s="56" t="str">
-        <x:f>IF(A39="","",IF(H39="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H39,"0.00")&amp;" citations per year. ")&amp;IF(I39="","Add total citations and publication year for the over-time comparison. ",IF(I39&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I39&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J39="","Name the benchmark and add its annual rate.",IF(J39&gt;1.1,"Against "&amp;F39&amp;": above the benchmark.",IF(J39&lt;0.9,"Against "&amp;F39&amp;": below the benchmark.","Against "&amp;F39&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A39="","",IF(H39="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H39,"0.00")&amp;" citations per year. ")&amp;IF(I39="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I39&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I39&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J39="","Name the benchmark and add its annual rate.",IF(J39&gt;1.1,"Now vs. "&amp;F39&amp;": above the benchmark.",IF(J39&lt;0.9,"Now vs. "&amp;F39&amp;": below the benchmark.","Now vs. "&amp;F39&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L39" s="57"/>
     </x:row>
@@ -1596,7 +1596,7 @@
         <x:f>IF(OR(A40="",D40="",E40="",F40="",G40="",E40&lt;=0,G40&lt;=0),"",IFERROR(D40/(G40*E40),""))</x:f>
       </x:c>
       <x:c r="K40" s="56" t="str">
-        <x:f>IF(A40="","",IF(H40="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H40,"0.00")&amp;" citations per year. ")&amp;IF(I40="","Add total citations and publication year for the over-time comparison. ",IF(I40&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I40&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J40="","Name the benchmark and add its annual rate.",IF(J40&gt;1.1,"Against "&amp;F40&amp;": above the benchmark.",IF(J40&lt;0.9,"Against "&amp;F40&amp;": below the benchmark.","Against "&amp;F40&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A40="","",IF(H40="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H40,"0.00")&amp;" citations per year. ")&amp;IF(I40="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I40&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I40&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J40="","Name the benchmark and add its annual rate.",IF(J40&gt;1.1,"Now vs. "&amp;F40&amp;": above the benchmark.",IF(J40&lt;0.9,"Now vs. "&amp;F40&amp;": below the benchmark.","Now vs. "&amp;F40&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L40" s="57"/>
     </x:row>
@@ -1618,7 +1618,7 @@
         <x:f>IF(OR(A41="",D41="",E41="",F41="",G41="",E41&lt;=0,G41&lt;=0),"",IFERROR(D41/(G41*E41),""))</x:f>
       </x:c>
       <x:c r="K41" s="56" t="str">
-        <x:f>IF(A41="","",IF(H41="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H41,"0.00")&amp;" citations per year. ")&amp;IF(I41="","Add total citations and publication year for the over-time comparison. ",IF(I41&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I41&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J41="","Name the benchmark and add its annual rate.",IF(J41&gt;1.1,"Against "&amp;F41&amp;": above the benchmark.",IF(J41&lt;0.9,"Against "&amp;F41&amp;": below the benchmark.","Against "&amp;F41&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A41="","",IF(H41="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H41,"0.00")&amp;" citations per year. ")&amp;IF(I41="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I41&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I41&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J41="","Name the benchmark and add its annual rate.",IF(J41&gt;1.1,"Now vs. "&amp;F41&amp;": above the benchmark.",IF(J41&lt;0.9,"Now vs. "&amp;F41&amp;": below the benchmark.","Now vs. "&amp;F41&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L41" s="57"/>
     </x:row>
@@ -1640,7 +1640,7 @@
         <x:f>IF(OR(A42="",D42="",E42="",F42="",G42="",E42&lt;=0,G42&lt;=0),"",IFERROR(D42/(G42*E42),""))</x:f>
       </x:c>
       <x:c r="K42" s="56" t="str">
-        <x:f>IF(A42="","",IF(H42="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H42,"0.00")&amp;" citations per year. ")&amp;IF(I42="","Add total citations and publication year for the over-time comparison. ",IF(I42&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I42&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J42="","Name the benchmark and add its annual rate.",IF(J42&gt;1.1,"Against "&amp;F42&amp;": above the benchmark.",IF(J42&lt;0.9,"Against "&amp;F42&amp;": below the benchmark.","Against "&amp;F42&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A42="","",IF(H42="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H42,"0.00")&amp;" citations per year. ")&amp;IF(I42="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I42&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I42&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J42="","Name the benchmark and add its annual rate.",IF(J42&gt;1.1,"Now vs. "&amp;F42&amp;": above the benchmark.",IF(J42&lt;0.9,"Now vs. "&amp;F42&amp;": below the benchmark.","Now vs. "&amp;F42&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L42" s="57"/>
     </x:row>
@@ -1662,7 +1662,7 @@
         <x:f>IF(OR(A43="",D43="",E43="",F43="",G43="",E43&lt;=0,G43&lt;=0),"",IFERROR(D43/(G43*E43),""))</x:f>
       </x:c>
       <x:c r="K43" s="56" t="str">
-        <x:f>IF(A43="","",IF(H43="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H43,"0.00")&amp;" citations per year. ")&amp;IF(I43="","Add total citations and publication year for the over-time comparison. ",IF(I43&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I43&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J43="","Name the benchmark and add its annual rate.",IF(J43&gt;1.1,"Against "&amp;F43&amp;": above the benchmark.",IF(J43&lt;0.9,"Against "&amp;F43&amp;": below the benchmark.","Against "&amp;F43&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A43="","",IF(H43="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H43,"0.00")&amp;" citations per year. ")&amp;IF(I43="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I43&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I43&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J43="","Name the benchmark and add its annual rate.",IF(J43&gt;1.1,"Now vs. "&amp;F43&amp;": above the benchmark.",IF(J43&lt;0.9,"Now vs. "&amp;F43&amp;": below the benchmark.","Now vs. "&amp;F43&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L43" s="57"/>
     </x:row>
@@ -1684,7 +1684,7 @@
         <x:f>IF(OR(A44="",D44="",E44="",F44="",G44="",E44&lt;=0,G44&lt;=0),"",IFERROR(D44/(G44*E44),""))</x:f>
       </x:c>
       <x:c r="K44" s="56" t="str">
-        <x:f>IF(A44="","",IF(H44="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H44,"0.00")&amp;" citations per year. ")&amp;IF(I44="","Add total citations and publication year for the over-time comparison. ",IF(I44&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I44&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J44="","Name the benchmark and add its annual rate.",IF(J44&gt;1.1,"Against "&amp;F44&amp;": above the benchmark.",IF(J44&lt;0.9,"Against "&amp;F44&amp;": below the benchmark.","Against "&amp;F44&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A44="","",IF(H44="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H44,"0.00")&amp;" citations per year. ")&amp;IF(I44="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I44&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I44&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J44="","Name the benchmark and add its annual rate.",IF(J44&gt;1.1,"Now vs. "&amp;F44&amp;": above the benchmark.",IF(J44&lt;0.9,"Now vs. "&amp;F44&amp;": below the benchmark.","Now vs. "&amp;F44&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L44" s="57"/>
     </x:row>
@@ -1706,7 +1706,7 @@
         <x:f>IF(OR(A45="",D45="",E45="",F45="",G45="",E45&lt;=0,G45&lt;=0),"",IFERROR(D45/(G45*E45),""))</x:f>
       </x:c>
       <x:c r="K45" s="56" t="str">
-        <x:f>IF(A45="","",IF(H45="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H45,"0.00")&amp;" citations per year. ")&amp;IF(I45="","Add total citations and publication year for the over-time comparison. ",IF(I45&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I45&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J45="","Name the benchmark and add its annual rate.",IF(J45&gt;1.1,"Against "&amp;F45&amp;": above the benchmark.",IF(J45&lt;0.9,"Against "&amp;F45&amp;": below the benchmark.","Against "&amp;F45&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A45="","",IF(H45="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H45,"0.00")&amp;" citations per year. ")&amp;IF(I45="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I45&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I45&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J45="","Name the benchmark and add its annual rate.",IF(J45&gt;1.1,"Now vs. "&amp;F45&amp;": above the benchmark.",IF(J45&lt;0.9,"Now vs. "&amp;F45&amp;": below the benchmark.","Now vs. "&amp;F45&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L45" s="57"/>
     </x:row>
@@ -1728,7 +1728,7 @@
         <x:f>IF(OR(A46="",D46="",E46="",F46="",G46="",E46&lt;=0,G46&lt;=0),"",IFERROR(D46/(G46*E46),""))</x:f>
       </x:c>
       <x:c r="K46" s="56" t="str">
-        <x:f>IF(A46="","",IF(H46="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H46,"0.00")&amp;" citations per year. ")&amp;IF(I46="","Add total citations and publication year for the over-time comparison. ",IF(I46&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I46&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J46="","Name the benchmark and add its annual rate.",IF(J46&gt;1.1,"Against "&amp;F46&amp;": above the benchmark.",IF(J46&lt;0.9,"Against "&amp;F46&amp;": below the benchmark.","Against "&amp;F46&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A46="","",IF(H46="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H46,"0.00")&amp;" citations per year. ")&amp;IF(I46="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I46&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I46&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J46="","Name the benchmark and add its annual rate.",IF(J46&gt;1.1,"Now vs. "&amp;F46&amp;": above the benchmark.",IF(J46&lt;0.9,"Now vs. "&amp;F46&amp;": below the benchmark.","Now vs. "&amp;F46&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L46" s="57"/>
     </x:row>
@@ -1750,7 +1750,7 @@
         <x:f>IF(OR(A47="",D47="",E47="",F47="",G47="",E47&lt;=0,G47&lt;=0),"",IFERROR(D47/(G47*E47),""))</x:f>
       </x:c>
       <x:c r="K47" s="56" t="str">
-        <x:f>IF(A47="","",IF(H47="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H47,"0.00")&amp;" citations per year. ")&amp;IF(I47="","Add total citations and publication year for the over-time comparison. ",IF(I47&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I47&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J47="","Name the benchmark and add its annual rate.",IF(J47&gt;1.1,"Against "&amp;F47&amp;": above the benchmark.",IF(J47&lt;0.9,"Against "&amp;F47&amp;": below the benchmark.","Against "&amp;F47&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A47="","",IF(H47="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H47,"0.00")&amp;" citations per year. ")&amp;IF(I47="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I47&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I47&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J47="","Name the benchmark and add its annual rate.",IF(J47&gt;1.1,"Now vs. "&amp;F47&amp;": above the benchmark.",IF(J47&lt;0.9,"Now vs. "&amp;F47&amp;": below the benchmark.","Now vs. "&amp;F47&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L47" s="57"/>
     </x:row>
@@ -1772,7 +1772,7 @@
         <x:f>IF(OR(A48="",D48="",E48="",F48="",G48="",E48&lt;=0,G48&lt;=0),"",IFERROR(D48/(G48*E48),""))</x:f>
       </x:c>
       <x:c r="K48" s="56" t="str">
-        <x:f>IF(A48="","",IF(H48="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H48,"0.00")&amp;" citations per year. ")&amp;IF(I48="","Add total citations and publication year for the over-time comparison. ",IF(I48&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I48&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J48="","Name the benchmark and add its annual rate.",IF(J48&gt;1.1,"Against "&amp;F48&amp;": above the benchmark.",IF(J48&lt;0.9,"Against "&amp;F48&amp;": below the benchmark.","Against "&amp;F48&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A48="","",IF(H48="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H48,"0.00")&amp;" citations per year. ")&amp;IF(I48="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I48&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I48&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J48="","Name the benchmark and add its annual rate.",IF(J48&gt;1.1,"Now vs. "&amp;F48&amp;": above the benchmark.",IF(J48&lt;0.9,"Now vs. "&amp;F48&amp;": below the benchmark.","Now vs. "&amp;F48&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L48" s="57"/>
     </x:row>
@@ -1794,7 +1794,7 @@
         <x:f>IF(OR(A49="",D49="",E49="",F49="",G49="",E49&lt;=0,G49&lt;=0),"",IFERROR(D49/(G49*E49),""))</x:f>
       </x:c>
       <x:c r="K49" s="56" t="str">
-        <x:f>IF(A49="","",IF(H49="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H49,"0.00")&amp;" citations per year. ")&amp;IF(I49="","Add total citations and publication year for the over-time comparison. ",IF(I49&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I49&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J49="","Name the benchmark and add its annual rate.",IF(J49&gt;1.1,"Against "&amp;F49&amp;": above the benchmark.",IF(J49&lt;0.9,"Against "&amp;F49&amp;": below the benchmark.","Against "&amp;F49&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A49="","",IF(H49="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H49,"0.00")&amp;" citations per year. ")&amp;IF(I49="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I49&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I49&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J49="","Name the benchmark and add its annual rate.",IF(J49&gt;1.1,"Now vs. "&amp;F49&amp;": above the benchmark.",IF(J49&lt;0.9,"Now vs. "&amp;F49&amp;": below the benchmark.","Now vs. "&amp;F49&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L49" s="57"/>
     </x:row>
@@ -1816,7 +1816,7 @@
         <x:f>IF(OR(A50="",D50="",E50="",F50="",G50="",E50&lt;=0,G50&lt;=0),"",IFERROR(D50/(G50*E50),""))</x:f>
       </x:c>
       <x:c r="K50" s="56" t="str">
-        <x:f>IF(A50="","",IF(H50="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H50,"0.00")&amp;" citations per year. ")&amp;IF(I50="","Add total citations and publication year for the over-time comparison. ",IF(I50&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I50&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J50="","Name the benchmark and add its annual rate.",IF(J50&gt;1.1,"Against "&amp;F50&amp;": above the benchmark.",IF(J50&lt;0.9,"Against "&amp;F50&amp;": below the benchmark.","Against "&amp;F50&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A50="","",IF(H50="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H50,"0.00")&amp;" citations per year. ")&amp;IF(I50="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I50&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I50&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J50="","Name the benchmark and add its annual rate.",IF(J50&gt;1.1,"Now vs. "&amp;F50&amp;": above the benchmark.",IF(J50&lt;0.9,"Now vs. "&amp;F50&amp;": below the benchmark.","Now vs. "&amp;F50&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L50" s="57"/>
     </x:row>
@@ -1838,7 +1838,7 @@
         <x:f>IF(OR(A51="",D51="",E51="",F51="",G51="",E51&lt;=0,G51&lt;=0),"",IFERROR(D51/(G51*E51),""))</x:f>
       </x:c>
       <x:c r="K51" s="56" t="str">
-        <x:f>IF(A51="","",IF(H51="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H51,"0.00")&amp;" citations per year. ")&amp;IF(I51="","Add total citations and publication year for the over-time comparison. ",IF(I51&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I51&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J51="","Name the benchmark and add its annual rate.",IF(J51&gt;1.1,"Against "&amp;F51&amp;": above the benchmark.",IF(J51&lt;0.9,"Against "&amp;F51&amp;": below the benchmark.","Against "&amp;F51&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A51="","",IF(H51="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H51,"0.00")&amp;" citations per year. ")&amp;IF(I51="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I51&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I51&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J51="","Name the benchmark and add its annual rate.",IF(J51&gt;1.1,"Now vs. "&amp;F51&amp;": above the benchmark.",IF(J51&lt;0.9,"Now vs. "&amp;F51&amp;": below the benchmark.","Now vs. "&amp;F51&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L51" s="57"/>
     </x:row>
@@ -1860,7 +1860,7 @@
         <x:f>IF(OR(A52="",D52="",E52="",F52="",G52="",E52&lt;=0,G52&lt;=0),"",IFERROR(D52/(G52*E52),""))</x:f>
       </x:c>
       <x:c r="K52" s="56" t="str">
-        <x:f>IF(A52="","",IF(H52="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H52,"0.00")&amp;" citations per year. ")&amp;IF(I52="","Add total citations and publication year for the over-time comparison. ",IF(I52&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I52&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J52="","Name the benchmark and add its annual rate.",IF(J52&gt;1.1,"Against "&amp;F52&amp;": above the benchmark.",IF(J52&lt;0.9,"Against "&amp;F52&amp;": below the benchmark.","Against "&amp;F52&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A52="","",IF(H52="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H52,"0.00")&amp;" citations per year. ")&amp;IF(I52="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I52&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I52&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J52="","Name the benchmark and add its annual rate.",IF(J52&gt;1.1,"Now vs. "&amp;F52&amp;": above the benchmark.",IF(J52&lt;0.9,"Now vs. "&amp;F52&amp;": below the benchmark.","Now vs. "&amp;F52&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L52" s="57"/>
     </x:row>
@@ -1882,7 +1882,7 @@
         <x:f>IF(OR(A53="",D53="",E53="",F53="",G53="",E53&lt;=0,G53&lt;=0),"",IFERROR(D53/(G53*E53),""))</x:f>
       </x:c>
       <x:c r="K53" s="56" t="str">
-        <x:f>IF(A53="","",IF(H53="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H53,"0.00")&amp;" citations per year. ")&amp;IF(I53="","Add total citations and publication year for the over-time comparison. ",IF(I53&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I53&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J53="","Name the benchmark and add its annual rate.",IF(J53&gt;1.1,"Against "&amp;F53&amp;": above the benchmark.",IF(J53&lt;0.9,"Against "&amp;F53&amp;": below the benchmark.","Against "&amp;F53&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A53="","",IF(H53="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H53,"0.00")&amp;" citations per year. ")&amp;IF(I53="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I53&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I53&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J53="","Name the benchmark and add its annual rate.",IF(J53&gt;1.1,"Now vs. "&amp;F53&amp;": above the benchmark.",IF(J53&lt;0.9,"Now vs. "&amp;F53&amp;": below the benchmark.","Now vs. "&amp;F53&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L53" s="57"/>
     </x:row>
@@ -1904,7 +1904,7 @@
         <x:f>IF(OR(A54="",D54="",E54="",F54="",G54="",E54&lt;=0,G54&lt;=0),"",IFERROR(D54/(G54*E54),""))</x:f>
       </x:c>
       <x:c r="K54" s="56" t="str">
-        <x:f>IF(A54="","",IF(H54="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H54,"0.00")&amp;" citations per year. ")&amp;IF(I54="","Add total citations and publication year for the over-time comparison. ",IF(I54&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I54&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J54="","Name the benchmark and add its annual rate.",IF(J54&gt;1.1,"Against "&amp;F54&amp;": above the benchmark.",IF(J54&lt;0.9,"Against "&amp;F54&amp;": below the benchmark.","Against "&amp;F54&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A54="","",IF(H54="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H54,"0.00")&amp;" citations per year. ")&amp;IF(I54="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I54&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I54&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J54="","Name the benchmark and add its annual rate.",IF(J54&gt;1.1,"Now vs. "&amp;F54&amp;": above the benchmark.",IF(J54&lt;0.9,"Now vs. "&amp;F54&amp;": below the benchmark.","Now vs. "&amp;F54&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L54" s="57"/>
     </x:row>
@@ -1926,7 +1926,7 @@
         <x:f>IF(OR(A55="",D55="",E55="",F55="",G55="",E55&lt;=0,G55&lt;=0),"",IFERROR(D55/(G55*E55),""))</x:f>
       </x:c>
       <x:c r="K55" s="56" t="str">
-        <x:f>IF(A55="","",IF(H55="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H55,"0.00")&amp;" citations per year. ")&amp;IF(I55="","Add total citations and publication year for the over-time comparison. ",IF(I55&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I55&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J55="","Name the benchmark and add its annual rate.",IF(J55&gt;1.1,"Against "&amp;F55&amp;": above the benchmark.",IF(J55&lt;0.9,"Against "&amp;F55&amp;": below the benchmark.","Against "&amp;F55&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A55="","",IF(H55="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H55,"0.00")&amp;" citations per year. ")&amp;IF(I55="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I55&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I55&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J55="","Name the benchmark and add its annual rate.",IF(J55&gt;1.1,"Now vs. "&amp;F55&amp;": above the benchmark.",IF(J55&lt;0.9,"Now vs. "&amp;F55&amp;": below the benchmark.","Now vs. "&amp;F55&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L55" s="57"/>
     </x:row>
@@ -1948,9 +1948,14 @@
         <x:f>IF(OR(A56="",D56="",E56="",F56="",G56="",E56&lt;=0,G56&lt;=0),"",IFERROR(D56/(G56*E56),""))</x:f>
       </x:c>
       <x:c r="K56" s="56" t="str">
-        <x:f>IF(A56="","",IF(H56="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H56,"0.00")&amp;" citations per year. ")&amp;IF(I56="","Add total citations and publication year for the over-time comparison. ",IF(I56&gt;1.1,"Over time: faster than the paper's lifetime rate. ",IF(I56&lt;0.9,"Over time: slower than the paper's lifetime rate. ","Over time: about the same as the paper's lifetime rate. ")))&amp;IF(J56="","Name the benchmark and add its annual rate.",IF(J56&gt;1.1,"Against "&amp;F56&amp;": above the benchmark.",IF(J56&lt;0.9,"Against "&amp;F56&amp;": below the benchmark.","Against "&amp;F56&amp;": about the same as the benchmark."))))</x:f>
+        <x:f>IF(A56="","",IF(H56="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H56,"0.00")&amp;" citations per year. ")&amp;IF(I56="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I56&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I56&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J56="","Name the benchmark and add its annual rate.",IF(J56&gt;1.1,"Now vs. "&amp;F56&amp;": above the benchmark.",IF(J56&lt;0.9,"Now vs. "&amp;F56&amp;": below the benchmark.","Now vs. "&amp;F56&amp;": about the same as the benchmark."))))</x:f>
       </x:c>
       <x:c r="L56" s="57"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="K57" t="str">
+        <x:f>IF(A57="","",IF(H57="","Enter the recent citations and number of recent years. ","Now: "&amp;TEXT(H57,"0.00")&amp;" citations per year. ")&amp;IF(I57="","Add total citations and publication year for the now-vs.-lifetime comparison. ",IF(I57&gt;1.1,"Now vs. lifetime: faster than the paper's lifetime rate. ",IF(I57&lt;0.9,"Now vs. lifetime: slower than the paper's lifetime rate. ","Now vs. lifetime: about the same as the paper's lifetime rate. ")))&amp;IF(J57="","Name the benchmark and add its annual rate.",IF(J57&gt;1.1,"Now vs. "&amp;F57&amp;": above the benchmark.",IF(J57&lt;0.9,"Now vs. "&amp;F57&amp;": below the benchmark.","Now vs. "&amp;F57&amp;": about the same as the benchmark."))))</x:f>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="63" t="str">
@@ -2010,7 +2015,7 @@
     </x:row>
     <x:row r="61" ht="34" customHeight="1">
       <x:c r="A61" s="70" t="str">
-        <x:v>Citations Per Year (Over Time)</x:v>
+        <x:v>Citations Per Year (Now vs. Lifetime)</x:v>
       </x:c>
       <x:c r="B61" s="70"/>
       <x:c r="C61" s="70"/>
@@ -2030,7 +2035,7 @@
     </x:row>
     <x:row r="62" ht="34" customHeight="1">
       <x:c r="A62" s="70" t="str">
-        <x:v>Citations Per Year (Against stated benchmark)</x:v>
+        <x:v>Citations Per Year (Now vs. Benchmark)</x:v>
       </x:c>
       <x:c r="B62" s="70"/>
       <x:c r="C62" s="70"/>
@@ -2107,7 +2112,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="8" t="str">
-        <x:v>Three results: Now, Over Time, and Against a named benchmark</x:v>
+        <x:v>Three results: Now, Now vs. Lifetime, and Now vs. Benchmark</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -2290,7 +2295,7 @@
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="74" t="str">
-        <x:v>Citations Per Year (Over Time)</x:v>
+        <x:v>Citations Per Year (Now vs. Lifetime)</x:v>
       </x:c>
       <x:c r="B22" s="74" t="str">
         <x:v>Recent rate: 5 per year. Lifetime rate: 10 per year. Result: 0.50.</x:v>
@@ -2301,7 +2306,7 @@
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="74" t="str">
-        <x:v>Citations Per Year (Against 2y-IF)</x:v>
+        <x:v>Citations Per Year (Now vs. Benchmark)</x:v>
       </x:c>
       <x:c r="B23" s="74" t="str">
         <x:v>Recent rate: 5 per year. Two-year impact factor: 3.0. Result: 1.67.</x:v>
@@ -2348,7 +2353,7 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="119" t="str">
-        <x:v>Grundy, F., &amp; Grundy, J. G. (under review). Citations per year now, over time, and against a benchmark: Transparent metrics for article-level impact. Calculator version 1.0 (July 28, 2026).</x:v>
+        <x:v>Grundy, F., &amp; Grundy, J. G. (under review). Transparent Metrics for Article-Level Impact Using Citations Per Year: Now, Now vs. Lifetime, and Now vs. Benchmark. Calculator version 1.0 (July 28, 2026).</x:v>
       </x:c>
       <x:c r="B32" s="120"/>
       <x:c r="C32" s="121"/>

</xml_diff>